<commit_message>
Raspberry con microSD de 64 GB en vez de NVMe
- Fuera el SSD y el M.2 HAT+ de las listas (total de compra 1.146,74 € + 41,40 $).
- Registros de los contenedores limitados (3 × 10 MB) para no desgastar la tarjeta.
- README de la Raspberry: tarjeta, límite del diario del sistema y copias fuera de la SD.
- Guía de instalación y plan actualizados.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RyhjygNwHjQbu5NjbwJkqd
</commit_message>
<xml_diff>
--- a/docs/07-lista-compra.xlsx
+++ b/docs/07-lista-compra.xlsx
@@ -443,8 +443,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I98"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:I96"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>SSD NVMe M.2 2242 256 GB Waveshare</t>
+          <t>Batería RTC oficial Raspberry Pi 5</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3517,11 +3517,11 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>https://www.kubii.com/es/medios-de-almacenamiento/4997-disco-duro-ssd-nvme-m2-2242-3272496325340.html</t>
+          <t>https://www.kubii.com/es/baterias-pilas/4110-bateria-rtc-para-raspberry-pi-5-5056561803739.html</t>
         </is>
       </c>
       <c r="F80" s="4" t="n">
-        <v>79.90000000000001</v>
+        <v>6</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -3532,11 +3532,7 @@
         <f>B80*F80</f>
         <v/>
       </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>El SSD oficial está agotado</t>
-        </is>
-      </c>
+      <c r="I80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3549,7 +3545,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Raspberry Pi M.2 HAT+ oficial</t>
+          <t>Fuente oficial Raspberry Pi 27 W USB-C</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3559,11 +3555,11 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>https://www.kubii.com/es/hat-dac-modulos/4114-m2-hat-para-raspberry-pi-5-5056561803463.html</t>
+          <t>https://www.kubii.com/es/fuentes-de-alimentacion/4107-1890-fuente-de-alimentacion-raspberry-pi-27w-usb-c-3272496315761.html</t>
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>14.1</v>
+        <v>12.9</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -3587,7 +3583,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Batería RTC oficial Raspberry Pi 5</t>
+          <t>Active Cooler oficial Raspberry Pi 5</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3597,7 +3593,7 @@
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>https://www.kubii.com/es/baterias-pilas/4110-bateria-rtc-para-raspberry-pi-5-5056561803739.html</t>
+          <t>https://www.kubii.com/es/ventiladores-disipadores-de-calor/4109-ventilador-disipador-para-raspberry-pi-5-5056561803357.html</t>
         </is>
       </c>
       <c r="F82" s="4" t="n">
@@ -3625,21 +3621,21 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Fuente oficial Raspberry Pi 27 W USB-C</t>
+          <t>Adaptador USB 3.0 a Ethernet Gigabit</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Kubii</t>
+          <t>Tiendatec</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>https://www.kubii.com/es/fuentes-de-alimentacion/4107-1890-fuente-de-alimentacion-raspberry-pi-27w-usb-c-3272496315761.html</t>
+          <t>https://www.tiendatec.es/maker-zone/comunicaciones-redes/2057-adaptador-usb-3-0-a-ethernet-gigabit-8436574700480.html</t>
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>12.9</v>
+        <v>12.95</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -3650,7 +3646,11 @@
         <f>B83*F83</f>
         <v/>
       </c>
-      <c r="I83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Pedir el de chip RTL8153</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3659,25 +3659,25 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Active Cooler oficial Raspberry Pi 5</t>
+          <t>Latiguillo UTP Cat6 1 m</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Kubii</t>
+          <t>Electrónica Embajadores</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>https://www.kubii.com/es/ventiladores-disipadores-de-calor/4109-ventilador-disipador-para-raspberry-pi-5-5056561803357.html</t>
+          <t>https://www.electronicaembajadores.com/es/Productos/Detalle/CX3A601/</t>
         </is>
       </c>
       <c r="F84" s="4" t="n">
-        <v>6</v>
+        <v>1.38</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3688,7 +3688,11 @@
         <f>B84*F84</f>
         <v/>
       </c>
-      <c r="I84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Raspberry-inyector PoE y red del instituto</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3701,21 +3705,21 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Adaptador USB 3.0 a Ethernet Gigabit</t>
+          <t>SAI Salicru SPS 500 ONE v2 (opcional)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Tiendatec</t>
+          <t>Discoazul</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>https://www.tiendatec.es/maker-zone/comunicaciones-redes/2057-adaptador-usb-3-0-a-ethernet-gigabit-8436574700480.html</t>
+          <t>https://www.discoazul.com/sai-linea-interactiva-salicru-sps-500-one-v2-500va-240w-2-schuko.html</t>
         </is>
       </c>
       <c r="F85" s="4" t="n">
-        <v>12.95</v>
+        <v>63.99</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -3728,36 +3732,36 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Pedir el de chip RTL8153</t>
+          <t>Opcional</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>5. Raspberry Pi 5 y red</t>
+          <t>6. Calibración y medida</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Latiguillo UTP Cat6 1 m</t>
+          <t>Solución tampón pH 4,01 Hanna 230 ml</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Electrónica Embajadores</t>
+          <t>Hanna Instruments</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>https://www.electronicaembajadores.com/es/Productos/Detalle/CX3A601/</t>
+          <t>https://www.hannainst.es/parametros/5096-solucion-tampon-ph-401.html</t>
         </is>
       </c>
       <c r="F86" s="4" t="n">
-        <v>1.38</v>
+        <v>12.1</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -3768,16 +3772,12 @@
         <f>B86*F86</f>
         <v/>
       </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>Raspberry-inyector PoE y red del instituto</t>
-        </is>
-      </c>
+      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>5. Raspberry Pi 5 y red</t>
+          <t>6. Calibración y medida</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -3785,21 +3785,21 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SAI Salicru SPS 500 ONE v2 (opcional)</t>
+          <t>Solución tampón pH 7,01 Hanna 230 ml</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Discoazul</t>
+          <t>Hanna Instruments</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>https://www.discoazul.com/sai-linea-interactiva-salicru-sps-500-one-v2-500va-240w-2-schuko.html</t>
+          <t>https://www.hannainst.es/parametros/5099-solucion-tampon-ph-701.html</t>
         </is>
       </c>
       <c r="F87" s="4" t="n">
-        <v>63.99</v>
+        <v>12.1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -3810,11 +3810,7 @@
         <f>B87*F87</f>
         <v/>
       </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>Opcional</t>
-        </is>
-      </c>
+      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3827,7 +3823,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Solución tampón pH 4,01 Hanna 230 ml</t>
+          <t>Solución tampón pH 10,01 Hanna 230 ml</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3837,7 +3833,7 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>https://www.hannainst.es/parametros/5096-solucion-tampon-ph-401.html</t>
+          <t>https://www.hannainst.es/parametros/5095-solucion-tampon-ph-1001.html</t>
         </is>
       </c>
       <c r="F88" s="4" t="n">
@@ -3865,7 +3861,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Solución tampón pH 7,01 Hanna 230 ml</t>
+          <t>Solución de almacenamiento de electrodos Hanna 230 ml</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3875,11 +3871,11 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>https://www.hannainst.es/parametros/5099-solucion-tampon-ph-701.html</t>
+          <t>https://www.hannainst.es/parametros/4974-solucion-almacenamiento-electrodos.html</t>
         </is>
       </c>
       <c r="F89" s="4" t="n">
-        <v>12.1</v>
+        <v>21.78</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -3899,25 +3895,25 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Solución tampón pH 10,01 Hanna 230 ml</t>
+          <t>Vaso de precipitado 100 ml borosilicato</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Hanna Instruments</t>
+          <t>Daselab</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>https://www.hannainst.es/parametros/5095-solucion-tampon-ph-1001.html</t>
+          <t>https://www.daselab.es/vasos-de-vidrio/198-vaso-precipitado-forma-baja-100-ml.html</t>
         </is>
       </c>
       <c r="F90" s="4" t="n">
-        <v>12.1</v>
+        <v>1.45</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -3941,21 +3937,21 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Solución de almacenamiento de electrodos Hanna 230 ml</t>
+          <t>Escobillón nº 40 (limpiar sondas)</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Hanna Instruments</t>
+          <t>Daselab</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>https://www.hannainst.es/parametros/4974-solucion-almacenamiento-electrodos.html</t>
+          <t>https://www.daselab.es/labware/3156-escobillon-n-40-ptubos-medianos.html</t>
         </is>
       </c>
       <c r="F91" s="4" t="n">
-        <v>21.78</v>
+        <v>1.4</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -3975,25 +3971,25 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Vaso de precipitado 100 ml borosilicato</t>
+          <t>Vatímetro DC jOY-it COM-VAO10020</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Daselab</t>
+          <t>Electrónica Embajadores</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>https://www.daselab.es/vasos-de-vidrio/198-vaso-precipitado-forma-baja-100-ml.html</t>
+          <t>https://www.electronicaembajadores.com/es/Productos/Detalle/IPDDAM5/</t>
         </is>
       </c>
       <c r="F92" s="4" t="n">
-        <v>1.45</v>
+        <v>14.9</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -4004,7 +4000,11 @@
         <f>B92*F92</f>
         <v/>
       </c>
-      <c r="I92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Medir consumos en la fase 6</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4017,127 +4017,47 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Escobillón nº 40 (limpiar sondas)</t>
+          <t>Agua destilada (garrafa 5 L)</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Daselab</t>
-        </is>
-      </c>
-      <c r="E93" s="3" t="inlineStr">
-        <is>
-          <t>https://www.daselab.es/labware/3156-escobillon-n-40-ptubos-medianos.html</t>
-        </is>
-      </c>
-      <c r="F93" s="4" t="n">
-        <v>1.4</v>
-      </c>
+          <t>Supermercado o ferretería</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" s="4" t="n"/>
       <c r="G93" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="H93" s="4">
-        <f>B93*F93</f>
-        <v/>
-      </c>
-      <c r="I93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>6. Calibración y medida</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
-        <v>1</v>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Vatímetro DC jOY-it COM-VAO10020</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Electrónica Embajadores</t>
-        </is>
-      </c>
-      <c r="E94" s="3" t="inlineStr">
-        <is>
-          <t>https://www.electronicaembajadores.com/es/Productos/Detalle/IPDDAM5/</t>
-        </is>
-      </c>
-      <c r="F94" s="4" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H94" s="4">
-        <f>B94*F94</f>
-        <v/>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>Medir consumos en la fase 6</t>
+      <c r="H93" s="4" t="n"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Compra local, unos 2 €</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>6. Calibración y medida</t>
-        </is>
-      </c>
-      <c r="B95" t="n">
-        <v>1</v>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Agua destilada (garrafa 5 L)</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>Supermercado o ferretería</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" s="4" t="n"/>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="n"/>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>Compra local, unos 2 €</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="G97" s="5" t="inlineStr">
+      <c r="G95" s="5" t="inlineStr">
         <is>
           <t>Total €</t>
         </is>
       </c>
-      <c r="H97" s="5">
-        <f>SUMIF(G5:G95,"EUR",H5:H95)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98">
-      <c r="G98" s="5" t="inlineStr">
+      <c r="H95" s="5">
+        <f>SUMIF(G5:G93,"EUR",H5:H93)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="G96" s="5" t="inlineStr">
         <is>
           <t>Total $</t>
         </is>
       </c>
-      <c r="H98" s="5">
-        <f>SUMIF(G5:G95,"USD",H5:H95)</f>
+      <c r="H96" s="5">
+        <f>SUMIF(G5:G93,"USD",H5:H93)</f>
         <v/>
       </c>
     </row>
@@ -4231,8 +4151,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lista de compra toda en euros con tiendas de España
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RyhjygNwHjQbu5NjbwJkqd
</commit_message>
<xml_diff>
--- a/docs/07-lista-compra.xlsx
+++ b/docs/07-lista-compra.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Precios con IVA salvo DFRobot (USD sin IVA). Enlaces comprobados el 29/09/2026.</t>
+          <t>Precios en euros con IVA. Enlaces comprobados el 29-30/09/2026.</t>
         </is>
       </c>
     </row>
@@ -529,25 +529,25 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ADC 16 bits I2C Gravity ADS1115 (DFR0553)</t>
+          <t>ADC 16 bits I2C ADS1115 Adafruit (STEMMA QT)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DFRobot (oficial)</t>
+          <t>Electrónica Embajadores</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://www.dfrobot.com/product-1730.html</t>
+          <t>https://www.electronicaembajadores.com/es/Productos/Detalle/LCINDD7/</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>15.5</v>
+        <v>21.63</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="H5" s="4">
@@ -556,7 +556,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Envío desde China; IVA y aduana aparte. Alternativa en España: Adafruit ADS1115 en Embajadores, 21,63 €: https://www.electronicaembajadores.com/es/Productos/Detalle/LCINDD7/</t>
+          <t>Mismo chip y dirección 0x48 (ADDR a GND); se conecta por pines a la placa base</t>
         </is>
       </c>
     </row>
@@ -571,25 +571,25 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Aislador de señal analógica Gravity (DFR0504)</t>
+          <t>Aislador de señal analógica Gravity DFRobot (DFR0504)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DFRobot (oficial)</t>
+          <t>Opencircuit</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://www.dfrobot.com/product-1621.html</t>
+          <t>https://opencircuit.es/producto/gravity-analog-signal-isolator</t>
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>19.9</v>
+        <v>29.5</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="H6" s="4">
@@ -598,7 +598,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>No lo vende ninguna tienda española comprobable</t>
+          <t>Trae 2 cables PH2.0. Tienda en español con precios en euros; envío a España desde 12,50 € (gratis desde 150 €)</t>
         </is>
       </c>
     </row>
@@ -638,11 +638,7 @@
         <f>B7*F7</f>
         <v/>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>En DFRobot cuesta 19,90 USD</t>
-        </is>
-      </c>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1198,32 +1194,36 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cables Gravity PH2.0 3 pines (pack) FIT0896</t>
+          <t>Cables Gravity PH2.0 3 pines a Dupont hembra, 50 cm (10 uds) FIT0769</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DFRobot (oficial)</t>
+          <t>Opencircuit</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://www.dfrobot.com/product-2552.html</t>
+          <t>https://opencircuit.es/producto/gravity-analog-sensor-cable-arduino-50cm-10</t>
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>6</v>
+        <v>4.6</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="H22" s="4">
         <f>B22*F22</f>
         <v/>
       </c>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Placa de pH y aislador a los pines de la placa base. Mismo pedido que el aislador</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4047,17 +4047,6 @@
       </c>
       <c r="H95" s="5">
         <f>SUMIF(G5:G93,"EUR",H5:H93)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96">
-      <c r="G96" s="5" t="inlineStr">
-        <is>
-          <t>Total $</t>
-        </is>
-      </c>
-      <c r="H96" s="5">
-        <f>SUMIF(G5:G93,"USD",H5:H93)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Red en la VLAN 500 del instituto: wAP 172.16.50.2 y Raspberry 172.16.50.3 con IP fija
- Un solo interfaz (eth0) con IP fija; fuera la red privada, el NAT y el adaptador USB-Ethernet.
- Datos de red en raspberry/red/red.env (los leen configurar-red.sh, firewall.sh e instalar.sh).
- Firewall por IP de origen: UDP 1700 y NTP solo desde el wAP.
- instalar.sh: si se entra por SSH con la IP del DHCP, prepara la red y pide reiniciar.
- Guías, prompts de Claude Code, configuración del wAP y lista de compra (sin adaptador USB: 1.189,52 €).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PWCmjiMrjRMb1Dx3k28GLJ
</commit_message>
<xml_diff>
--- a/docs/07-lista-compra.xlsx
+++ b/docs/07-lista-compra.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Compra" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compra" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,8 +443,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I95"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:I94"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -638,7 +638,6 @@
         <f>B7*F7</f>
         <v/>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -676,7 +675,6 @@
         <f>B8*F8</f>
         <v/>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -793,7 +791,6 @@
         <f>B11*F11</f>
         <v/>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -831,7 +828,6 @@
         <f>B12*F12</f>
         <v/>
       </c>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -911,7 +907,6 @@
         <f>B14*F14</f>
         <v/>
       </c>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -949,7 +944,6 @@
         <f>B15*F15</f>
         <v/>
       </c>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1029,7 +1023,6 @@
         <f>B17*F17</f>
         <v/>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1067,7 +1060,6 @@
         <f>B18*F18</f>
         <v/>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1105,7 +1097,6 @@
         <f>B19*F19</f>
         <v/>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1143,7 +1134,6 @@
         <f>B20*F20</f>
         <v/>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1181,7 +1171,6 @@
         <f>B21*F21</f>
         <v/>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1261,7 +1250,6 @@
         <f>B23*F23</f>
         <v/>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1383,7 +1371,6 @@
         <f>B26*F26</f>
         <v/>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1542,7 +1529,6 @@
         <f>B30*F30</f>
         <v/>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1622,7 +1608,6 @@
         <f>B32*F32</f>
         <v/>
       </c>
-      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1702,7 +1687,6 @@
         <f>B34*F34</f>
         <v/>
       </c>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1782,7 +1766,6 @@
         <f>B36*F36</f>
         <v/>
       </c>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1820,7 +1803,6 @@
         <f>B37*F37</f>
         <v/>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1984,7 +1966,6 @@
         <f>B41*F41</f>
         <v/>
       </c>
-      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2222,7 +2203,6 @@
         <f>B47*F47</f>
         <v/>
       </c>
-      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2260,7 +2240,6 @@
         <f>B48*F48</f>
         <v/>
       </c>
-      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2340,7 +2319,6 @@
         <f>B50*F50</f>
         <v/>
       </c>
-      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2378,7 +2356,6 @@
         <f>B51*F51</f>
         <v/>
       </c>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2416,7 +2393,6 @@
         <f>B52*F52</f>
         <v/>
       </c>
-      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2454,7 +2430,6 @@
         <f>B53*F53</f>
         <v/>
       </c>
-      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2534,7 +2509,6 @@
         <f>B55*F55</f>
         <v/>
       </c>
-      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2614,7 +2588,6 @@
         <f>B57*F57</f>
         <v/>
       </c>
-      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2694,7 +2667,6 @@
         <f>B59*F59</f>
         <v/>
       </c>
-      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2732,7 +2704,6 @@
         <f>B60*F60</f>
         <v/>
       </c>
-      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2770,7 +2741,6 @@
         <f>B61*F61</f>
         <v/>
       </c>
-      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2808,7 +2778,6 @@
         <f>B62*F62</f>
         <v/>
       </c>
-      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3140,7 +3109,6 @@
         <f>B70*F70</f>
         <v/>
       </c>
-      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3220,7 +3188,6 @@
         <f>B72*F72</f>
         <v/>
       </c>
-      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3258,7 +3225,6 @@
         <f>B73*F73</f>
         <v/>
       </c>
-      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3296,7 +3262,6 @@
         <f>B74*F74</f>
         <v/>
       </c>
-      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3334,7 +3299,6 @@
         <f>B75*F75</f>
         <v/>
       </c>
-      <c r="I75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3414,7 +3378,6 @@
         <f>B77*F77</f>
         <v/>
       </c>
-      <c r="I77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3494,7 +3457,6 @@
         <f>B79*F79</f>
         <v/>
       </c>
-      <c r="I79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3532,7 +3494,6 @@
         <f>B80*F80</f>
         <v/>
       </c>
-      <c r="I80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3570,7 +3531,6 @@
         <f>B81*F81</f>
         <v/>
       </c>
-      <c r="I81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3608,7 +3568,6 @@
         <f>B82*F82</f>
         <v/>
       </c>
-      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3617,25 +3576,25 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Adaptador USB 3.0 a Ethernet Gigabit</t>
+          <t>Latiguillo UTP Cat6 1 m</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Tiendatec</t>
+          <t>Electrónica Embajadores</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>https://www.tiendatec.es/maker-zone/comunicaciones-redes/2057-adaptador-usb-3-0-a-ethernet-gigabit-8436574700480.html</t>
+          <t>https://www.electronicaembajadores.com/es/Productos/Detalle/CX3A601/</t>
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>12.95</v>
+        <v>1.38</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -3648,7 +3607,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Pedir el de chip RTL8153</t>
+          <t>Raspberry → switch (VLAN 500) e inyector PoE → switch</t>
         </is>
       </c>
     </row>
@@ -3659,25 +3618,25 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Latiguillo UTP Cat6 1 m</t>
+          <t>SAI Salicru SPS 500 ONE v2 (opcional)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Electrónica Embajadores</t>
+          <t>Discoazul</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>https://www.electronicaembajadores.com/es/Productos/Detalle/CX3A601/</t>
+          <t>https://www.discoazul.com/sai-linea-interactiva-salicru-sps-500-one-v2-500va-240w-2-schuko.html</t>
         </is>
       </c>
       <c r="F84" s="4" t="n">
-        <v>1.38</v>
+        <v>63.99</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3690,14 +3649,14 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Raspberry-inyector PoE y red del instituto</t>
+          <t>Opcional</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>5. Raspberry Pi 5 y red</t>
+          <t>6. Calibración y medida</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -3705,21 +3664,21 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>SAI Salicru SPS 500 ONE v2 (opcional)</t>
+          <t>Solución tampón pH 4,01 Hanna 230 ml</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Discoazul</t>
+          <t>Hanna Instruments</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>https://www.discoazul.com/sai-linea-interactiva-salicru-sps-500-one-v2-500va-240w-2-schuko.html</t>
+          <t>https://www.hannainst.es/parametros/5096-solucion-tampon-ph-401.html</t>
         </is>
       </c>
       <c r="F85" s="4" t="n">
-        <v>63.99</v>
+        <v>12.1</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -3730,11 +3689,6 @@
         <f>B85*F85</f>
         <v/>
       </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>Opcional</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3747,7 +3701,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Solución tampón pH 4,01 Hanna 230 ml</t>
+          <t>Solución tampón pH 7,01 Hanna 230 ml</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3757,7 +3711,7 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>https://www.hannainst.es/parametros/5096-solucion-tampon-ph-401.html</t>
+          <t>https://www.hannainst.es/parametros/5099-solucion-tampon-ph-701.html</t>
         </is>
       </c>
       <c r="F86" s="4" t="n">
@@ -3772,7 +3726,6 @@
         <f>B86*F86</f>
         <v/>
       </c>
-      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3785,7 +3738,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Solución tampón pH 7,01 Hanna 230 ml</t>
+          <t>Solución tampón pH 10,01 Hanna 230 ml</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3795,7 +3748,7 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>https://www.hannainst.es/parametros/5099-solucion-tampon-ph-701.html</t>
+          <t>https://www.hannainst.es/parametros/5095-solucion-tampon-ph-1001.html</t>
         </is>
       </c>
       <c r="F87" s="4" t="n">
@@ -3810,7 +3763,6 @@
         <f>B87*F87</f>
         <v/>
       </c>
-      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3823,7 +3775,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Solución tampón pH 10,01 Hanna 230 ml</t>
+          <t>Solución de almacenamiento de electrodos Hanna 230 ml</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3833,11 +3785,11 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>https://www.hannainst.es/parametros/5095-solucion-tampon-ph-1001.html</t>
+          <t>https://www.hannainst.es/parametros/4974-solucion-almacenamiento-electrodos.html</t>
         </is>
       </c>
       <c r="F88" s="4" t="n">
-        <v>12.1</v>
+        <v>21.78</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -3848,7 +3800,6 @@
         <f>B88*F88</f>
         <v/>
       </c>
-      <c r="I88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3857,25 +3808,25 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Solución de almacenamiento de electrodos Hanna 230 ml</t>
+          <t>Vaso de precipitado 100 ml borosilicato</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Hanna Instruments</t>
+          <t>Daselab</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>https://www.hannainst.es/parametros/4974-solucion-almacenamiento-electrodos.html</t>
+          <t>https://www.daselab.es/vasos-de-vidrio/198-vaso-precipitado-forma-baja-100-ml.html</t>
         </is>
       </c>
       <c r="F89" s="4" t="n">
-        <v>21.78</v>
+        <v>1.45</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -3886,7 +3837,6 @@
         <f>B89*F89</f>
         <v/>
       </c>
-      <c r="I89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3895,11 +3845,11 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Vaso de precipitado 100 ml borosilicato</t>
+          <t>Escobillón nº 40 (limpiar sondas)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3909,11 +3859,11 @@
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>https://www.daselab.es/vasos-de-vidrio/198-vaso-precipitado-forma-baja-100-ml.html</t>
+          <t>https://www.daselab.es/labware/3156-escobillon-n-40-ptubos-medianos.html</t>
         </is>
       </c>
       <c r="F90" s="4" t="n">
-        <v>1.45</v>
+        <v>1.4</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -3924,7 +3874,6 @@
         <f>B90*F90</f>
         <v/>
       </c>
-      <c r="I90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3937,21 +3886,21 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Escobillón nº 40 (limpiar sondas)</t>
+          <t>Vatímetro DC jOY-it COM-VAO10020</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Daselab</t>
+          <t>Electrónica Embajadores</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>https://www.daselab.es/labware/3156-escobillon-n-40-ptubos-medianos.html</t>
+          <t>https://www.electronicaembajadores.com/es/Productos/Detalle/IPDDAM5/</t>
         </is>
       </c>
       <c r="F91" s="4" t="n">
-        <v>1.4</v>
+        <v>14.9</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -3962,7 +3911,11 @@
         <f>B91*F91</f>
         <v/>
       </c>
-      <c r="I91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Medir consumos en la fase 6</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3975,78 +3928,36 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Vatímetro DC jOY-it COM-VAO10020</t>
+          <t>Agua destilada (garrafa 5 L)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Electrónica Embajadores</t>
-        </is>
-      </c>
-      <c r="E92" s="3" t="inlineStr">
-        <is>
-          <t>https://www.electronicaembajadores.com/es/Productos/Detalle/IPDDAM5/</t>
-        </is>
-      </c>
-      <c r="F92" s="4" t="n">
-        <v>14.9</v>
-      </c>
+          <t>Supermercado o ferretería</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="n"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="H92" s="4">
-        <f>B92*F92</f>
-        <v/>
-      </c>
+      <c r="H92" s="4" t="n"/>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Medir consumos en la fase 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>6. Calibración y medida</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
-        <v>1</v>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Agua destilada (garrafa 5 L)</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>Supermercado o ferretería</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" s="4" t="n"/>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="H93" s="4" t="n"/>
-      <c r="I93" t="inlineStr">
-        <is>
           <t>Compra local, unos 2 €</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="G95" s="5" t="inlineStr">
+    <row r="93"/>
+    <row r="94">
+      <c r="G94" s="5" t="inlineStr">
         <is>
           <t>Total €</t>
         </is>
       </c>
-      <c r="H95" s="5">
-        <f>SUMIF(G5:G93,"EUR",H5:H93)</f>
+      <c r="H94" s="5">
+        <f>SUMIF(G5:G92,"EUR",H5:H92)</f>
         <v/>
       </c>
     </row>
@@ -4130,16 +4041,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId87"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>